<commit_message>
Power cards should be done now.
This should be the last power card.  Need to do one last review, but routing seems to be good.
</commit_message>
<xml_diff>
--- a/Lasser_Driver_v5/pm1p8V_pm5V_5Vref_5Vlaser/pm1p8V_pm5V_5Vref_5Vlaser_BOM_digikey.xlsx
+++ b/Lasser_Driver_v5/pm1p8V_pm5V_5Vref_5Vlaser/pm1p8V_pm5V_5Vref_5Vlaser_BOM_digikey.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E39"/>
+  <dimension ref="A1:E40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1393,6 +1393,31 @@
         </is>
       </c>
     </row>
+    <row r="40">
+      <c r="A40" t="n">
+        <v>2</v>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>ERJ-6BWFR020V</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>Panasonic Industry</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>R42, R43</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>20m 1%</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>